<commit_message>
Some graphs working and new enb counting strategy (to test)
</commit_message>
<xml_diff>
--- a/Functions/Images/disaster_percentage_0/micro_power_30/enb_data.xlsx
+++ b/Functions/Images/disaster_percentage_0/micro_power_30/enb_data.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,25 +462,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>RBs</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>min_snr_used</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>repetition</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>inifile</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>NumEnbs</t>
         </is>
@@ -497,24 +502,29 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="F2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>4.7</v>
+      <c r="H2" t="n">
+        <v>4.416666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -523,13 +533,14 @@
       <c r="C3" s="1" t="n"/>
       <c r="D3" s="1" t="n"/>
       <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>4.7</v>
+      <c r="H3" t="n">
+        <v>4.583333333333333</v>
       </c>
     </row>
     <row r="4">
@@ -538,13 +549,14 @@
       <c r="C4" s="1" t="n"/>
       <c r="D4" s="1" t="n"/>
       <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>5.1</v>
+      <c r="H4" t="n">
+        <v>5.416666666666667</v>
       </c>
     </row>
     <row r="5">
@@ -553,13 +565,14 @@
       <c r="C5" s="1" t="n"/>
       <c r="D5" s="1" t="n"/>
       <c r="E5" s="1" t="n"/>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>5</v>
+      <c r="H5" t="n">
+        <v>5.416666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -568,13 +581,14 @@
       <c r="C6" s="1" t="n"/>
       <c r="D6" s="1" t="n"/>
       <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>5.3</v>
+      <c r="H6" t="n">
+        <v>5.25</v>
       </c>
     </row>
     <row r="7">
@@ -583,13 +597,14 @@
       <c r="C7" s="1" t="n"/>
       <c r="D7" s="1" t="n"/>
       <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>4.7</v>
+      <c r="H7" t="n">
+        <v>4.75</v>
       </c>
     </row>
     <row r="8">
@@ -598,13 +613,14 @@
       <c r="C8" s="1" t="n"/>
       <c r="D8" s="1" t="n"/>
       <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>4.7</v>
+      <c r="H8" t="n">
+        <v>4.75</v>
       </c>
     </row>
     <row r="9">
@@ -613,13 +629,14 @@
       <c r="C9" s="1" t="n"/>
       <c r="D9" s="1" t="n"/>
       <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>4.6</v>
+      <c r="H9" t="n">
+        <v>4.666666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -628,13 +645,14 @@
       <c r="C10" s="1" t="n"/>
       <c r="D10" s="1" t="n"/>
       <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>4.7</v>
+      <c r="H10" t="n">
+        <v>4.75</v>
       </c>
     </row>
     <row r="11">
@@ -643,34 +661,36 @@
       <c r="C11" s="1" t="n"/>
       <c r="D11" s="1" t="n"/>
       <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_fixed_sliced_10.ini</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>4.3</v>
+      <c r="H11" t="n">
+        <v>4.416666666666667</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="1" t="n"/>
       <c r="C12" s="1" t="n"/>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="F12" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G12" t="n">
-        <v>7.2</v>
+      <c r="H12" t="n">
+        <v>6.916666666666667</v>
       </c>
     </row>
     <row r="13">
@@ -679,13 +699,14 @@
       <c r="C13" s="1" t="n"/>
       <c r="D13" s="1" t="n"/>
       <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>7.2</v>
+      <c r="H13" t="n">
+        <v>7.166666666666667</v>
       </c>
     </row>
     <row r="14">
@@ -694,13 +715,14 @@
       <c r="C14" s="1" t="n"/>
       <c r="D14" s="1" t="n"/>
       <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G14" t="n">
-        <v>7</v>
+      <c r="H14" t="n">
+        <v>7.25</v>
       </c>
     </row>
     <row r="15">
@@ -709,13 +731,14 @@
       <c r="C15" s="1" t="n"/>
       <c r="D15" s="1" t="n"/>
       <c r="E15" s="1" t="n"/>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F15" s="1" t="n"/>
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>7.6</v>
+      <c r="H15" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -724,13 +747,14 @@
       <c r="C16" s="1" t="n"/>
       <c r="D16" s="1" t="n"/>
       <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F16" s="1" t="n"/>
+      <c r="G16" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G16" t="n">
-        <v>7.4</v>
+      <c r="H16" t="n">
+        <v>7.083333333333333</v>
       </c>
     </row>
     <row r="17">
@@ -739,13 +763,14 @@
       <c r="C17" s="1" t="n"/>
       <c r="D17" s="1" t="n"/>
       <c r="E17" s="1" t="n"/>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F17" s="1" t="n"/>
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>7.4</v>
+      <c r="H17" t="n">
+        <v>7.25</v>
       </c>
     </row>
     <row r="18">
@@ -754,13 +779,14 @@
       <c r="C18" s="1" t="n"/>
       <c r="D18" s="1" t="n"/>
       <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F18" s="1" t="n"/>
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G18" t="n">
-        <v>7.3</v>
+      <c r="H18" t="n">
+        <v>7.333333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -769,13 +795,14 @@
       <c r="C19" s="1" t="n"/>
       <c r="D19" s="1" t="n"/>
       <c r="E19" s="1" t="n"/>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F19" s="1" t="n"/>
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G19" t="n">
-        <v>7.1</v>
+      <c r="H19" t="n">
+        <v>7.166666666666667</v>
       </c>
     </row>
     <row r="20">
@@ -784,13 +811,14 @@
       <c r="C20" s="1" t="n"/>
       <c r="D20" s="1" t="n"/>
       <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F20" s="1" t="n"/>
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G20" t="n">
-        <v>7.4</v>
+      <c r="H20" t="n">
+        <v>7.333333333333333</v>
       </c>
     </row>
     <row r="21">
@@ -799,34 +827,36 @@
       <c r="C21" s="1" t="n"/>
       <c r="D21" s="1" t="n"/>
       <c r="E21" s="1" t="n"/>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F21" s="1" t="n"/>
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_fixed_sliced_15.ini</t>
         </is>
       </c>
-      <c r="G21" t="n">
-        <v>6.9</v>
+      <c r="H21" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="1" t="n"/>
       <c r="C22" s="1" t="n"/>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D22" s="1" t="n"/>
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="F22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="G22" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G22" t="n">
-        <v>3.7</v>
+      <c r="H22" t="n">
+        <v>3.5</v>
       </c>
     </row>
     <row r="23">
@@ -835,13 +865,14 @@
       <c r="C23" s="1" t="n"/>
       <c r="D23" s="1" t="n"/>
       <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F23" s="1" t="n"/>
+      <c r="G23" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G23" t="n">
-        <v>3.7</v>
+      <c r="H23" t="n">
+        <v>3.666666666666667</v>
       </c>
     </row>
     <row r="24">
@@ -850,13 +881,14 @@
       <c r="C24" s="1" t="n"/>
       <c r="D24" s="1" t="n"/>
       <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F24" s="1" t="n"/>
+      <c r="G24" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G24" t="n">
-        <v>3.2</v>
+      <c r="H24" t="n">
+        <v>3.583333333333333</v>
       </c>
     </row>
     <row r="25">
@@ -865,13 +897,14 @@
       <c r="C25" s="1" t="n"/>
       <c r="D25" s="1" t="n"/>
       <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F25" s="1" t="n"/>
+      <c r="G25" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G25" t="n">
-        <v>3.6</v>
+      <c r="H25" t="n">
+        <v>3.666666666666667</v>
       </c>
     </row>
     <row r="26">
@@ -880,13 +913,14 @@
       <c r="C26" s="1" t="n"/>
       <c r="D26" s="1" t="n"/>
       <c r="E26" s="1" t="n"/>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F26" s="1" t="n"/>
+      <c r="G26" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G26" t="n">
-        <v>3.7</v>
+      <c r="H26" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="27">
@@ -895,13 +929,14 @@
       <c r="C27" s="1" t="n"/>
       <c r="D27" s="1" t="n"/>
       <c r="E27" s="1" t="n"/>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G27" t="n">
-        <v>3.6</v>
+      <c r="H27" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="28">
@@ -910,13 +945,14 @@
       <c r="C28" s="1" t="n"/>
       <c r="D28" s="1" t="n"/>
       <c r="E28" s="1" t="n"/>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F28" s="1" t="n"/>
+      <c r="G28" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G28" t="n">
-        <v>3.8</v>
+      <c r="H28" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="29">
@@ -925,13 +961,14 @@
       <c r="C29" s="1" t="n"/>
       <c r="D29" s="1" t="n"/>
       <c r="E29" s="1" t="n"/>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F29" s="1" t="n"/>
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G29" t="n">
-        <v>3.6</v>
+      <c r="H29" t="n">
+        <v>3.666666666666667</v>
       </c>
     </row>
     <row r="30">
@@ -940,13 +977,14 @@
       <c r="C30" s="1" t="n"/>
       <c r="D30" s="1" t="n"/>
       <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F30" s="1" t="n"/>
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G30" t="n">
-        <v>3.7</v>
+      <c r="H30" t="n">
+        <v>3.666666666666667</v>
       </c>
     </row>
     <row r="31">
@@ -955,19 +993,20 @@
       <c r="C31" s="1" t="n"/>
       <c r="D31" s="1" t="n"/>
       <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F31" s="1" t="n"/>
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_fixed_sliced_5.ini</t>
         </is>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
         <v>3.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>Ga</t>
         </is>
       </c>
       <c r="B32" s="1" t="n">
@@ -975,24 +1014,29 @@
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="F32" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>4.8</v>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>7.083333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -1001,13 +1045,14 @@
       <c r="C33" s="1" t="n"/>
       <c r="D33" s="1" t="n"/>
       <c r="E33" s="1" t="n"/>
-      <c r="F33" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>3.9</v>
+      <c r="F33" s="1" t="n"/>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>7.5</v>
       </c>
     </row>
     <row r="34">
@@ -1016,13 +1061,14 @@
       <c r="C34" s="1" t="n"/>
       <c r="D34" s="1" t="n"/>
       <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>4.7</v>
+      <c r="F34" s="1" t="n"/>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>10.58333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -1031,13 +1077,14 @@
       <c r="C35" s="1" t="n"/>
       <c r="D35" s="1" t="n"/>
       <c r="E35" s="1" t="n"/>
-      <c r="F35" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>4.6</v>
+      <c r="F35" s="1" t="n"/>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="36">
@@ -1046,13 +1093,14 @@
       <c r="C36" s="1" t="n"/>
       <c r="D36" s="1" t="n"/>
       <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>4.7</v>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>6.583333333333333</v>
       </c>
     </row>
     <row r="37">
@@ -1061,13 +1109,14 @@
       <c r="C37" s="1" t="n"/>
       <c r="D37" s="1" t="n"/>
       <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>3.9</v>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>5.75</v>
       </c>
     </row>
     <row r="38">
@@ -1076,13 +1125,14 @@
       <c r="C38" s="1" t="n"/>
       <c r="D38" s="1" t="n"/>
       <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>3.7</v>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="39">
@@ -1091,13 +1141,14 @@
       <c r="C39" s="1" t="n"/>
       <c r="D39" s="1" t="n"/>
       <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>4.7</v>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>8.833333333333334</v>
       </c>
     </row>
     <row r="40">
@@ -1106,13 +1157,14 @@
       <c r="C40" s="1" t="n"/>
       <c r="D40" s="1" t="n"/>
       <c r="E40" s="1" t="n"/>
-      <c r="F40" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>3.7</v>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>7.833333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -1121,34 +1173,36 @@
       <c r="C41" s="1" t="n"/>
       <c r="D41" s="1" t="n"/>
       <c r="E41" s="1" t="n"/>
-      <c r="F41" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_single_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>3.7</v>
+      <c r="F41" s="1" t="n"/>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_ga_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>8.666666666666666</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n"/>
       <c r="B42" s="1" t="n"/>
       <c r="C42" s="1" t="n"/>
-      <c r="D42" s="1" t="inlineStr">
+      <c r="D42" s="1" t="n"/>
+      <c r="E42" s="1" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="F42" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F42" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>6.8</v>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>14.41666666666667</v>
       </c>
     </row>
     <row r="43">
@@ -1157,13 +1211,14 @@
       <c r="C43" s="1" t="n"/>
       <c r="D43" s="1" t="n"/>
       <c r="E43" s="1" t="n"/>
-      <c r="F43" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>6.6</v>
+      <c r="F43" s="1" t="n"/>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>15.33333333333333</v>
       </c>
     </row>
     <row r="44">
@@ -1172,13 +1227,14 @@
       <c r="C44" s="1" t="n"/>
       <c r="D44" s="1" t="n"/>
       <c r="E44" s="1" t="n"/>
-      <c r="F44" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>6.4</v>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>18.83333333333333</v>
       </c>
     </row>
     <row r="45">
@@ -1187,13 +1243,14 @@
       <c r="C45" s="1" t="n"/>
       <c r="D45" s="1" t="n"/>
       <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>6.6</v>
+      <c r="F45" s="1" t="n"/>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>15.75</v>
       </c>
     </row>
     <row r="46">
@@ -1202,13 +1259,14 @@
       <c r="C46" s="1" t="n"/>
       <c r="D46" s="1" t="n"/>
       <c r="E46" s="1" t="n"/>
-      <c r="F46" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>6.4</v>
+      <c r="F46" s="1" t="n"/>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>19.91666666666667</v>
       </c>
     </row>
     <row r="47">
@@ -1217,13 +1275,14 @@
       <c r="C47" s="1" t="n"/>
       <c r="D47" s="1" t="n"/>
       <c r="E47" s="1" t="n"/>
-      <c r="F47" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>5.6</v>
+      <c r="F47" s="1" t="n"/>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>15.83333333333333</v>
       </c>
     </row>
     <row r="48">
@@ -1232,13 +1291,14 @@
       <c r="C48" s="1" t="n"/>
       <c r="D48" s="1" t="n"/>
       <c r="E48" s="1" t="n"/>
-      <c r="F48" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>6.5</v>
+      <c r="F48" s="1" t="n"/>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="49">
@@ -1247,13 +1307,14 @@
       <c r="C49" s="1" t="n"/>
       <c r="D49" s="1" t="n"/>
       <c r="E49" s="1" t="n"/>
-      <c r="F49" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>6.5</v>
+      <c r="F49" s="1" t="n"/>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>8.583333333333334</v>
       </c>
     </row>
     <row r="50">
@@ -1262,13 +1323,14 @@
       <c r="C50" s="1" t="n"/>
       <c r="D50" s="1" t="n"/>
       <c r="E50" s="1" t="n"/>
-      <c r="F50" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>5.5</v>
+      <c r="F50" s="1" t="n"/>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>9.416666666666666</v>
       </c>
     </row>
     <row r="51">
@@ -1277,34 +1339,36 @@
       <c r="C51" s="1" t="n"/>
       <c r="D51" s="1" t="n"/>
       <c r="E51" s="1" t="n"/>
-      <c r="F51" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_single_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>6.5</v>
+      <c r="F51" s="1" t="n"/>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_ga_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>14.75</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n"/>
       <c r="B52" s="1" t="n"/>
       <c r="C52" s="1" t="n"/>
-      <c r="D52" s="1" t="inlineStr">
+      <c r="D52" s="1" t="n"/>
+      <c r="E52" s="1" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E52" s="1" t="n">
+      <c r="F52" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>2.9</v>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>4.416666666666667</v>
       </c>
     </row>
     <row r="53">
@@ -1313,13 +1377,14 @@
       <c r="C53" s="1" t="n"/>
       <c r="D53" s="1" t="n"/>
       <c r="E53" s="1" t="n"/>
-      <c r="F53" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>3</v>
+      <c r="F53" s="1" t="n"/>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>4.083333333333333</v>
       </c>
     </row>
     <row r="54">
@@ -1328,13 +1393,14 @@
       <c r="C54" s="1" t="n"/>
       <c r="D54" s="1" t="n"/>
       <c r="E54" s="1" t="n"/>
-      <c r="F54" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>3.8</v>
+      <c r="F54" s="1" t="n"/>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>6.666666666666667</v>
       </c>
     </row>
     <row r="55">
@@ -1343,13 +1409,14 @@
       <c r="C55" s="1" t="n"/>
       <c r="D55" s="1" t="n"/>
       <c r="E55" s="1" t="n"/>
-      <c r="F55" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>3.7</v>
+      <c r="F55" s="1" t="n"/>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="56">
@@ -1358,13 +1425,14 @@
       <c r="C56" s="1" t="n"/>
       <c r="D56" s="1" t="n"/>
       <c r="E56" s="1" t="n"/>
-      <c r="F56" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>2.9</v>
+      <c r="F56" s="1" t="n"/>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>4.583333333333333</v>
       </c>
     </row>
     <row r="57">
@@ -1373,13 +1441,14 @@
       <c r="C57" s="1" t="n"/>
       <c r="D57" s="1" t="n"/>
       <c r="E57" s="1" t="n"/>
-      <c r="F57" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>3.8</v>
+      <c r="F57" s="1" t="n"/>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>4.333333333333333</v>
       </c>
     </row>
     <row r="58">
@@ -1388,13 +1457,14 @@
       <c r="C58" s="1" t="n"/>
       <c r="D58" s="1" t="n"/>
       <c r="E58" s="1" t="n"/>
-      <c r="F58" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>3.7</v>
+      <c r="F58" s="1" t="n"/>
+      <c r="G58" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="59">
@@ -1403,13 +1473,14 @@
       <c r="C59" s="1" t="n"/>
       <c r="D59" s="1" t="n"/>
       <c r="E59" s="1" t="n"/>
-      <c r="F59" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G59" t="n">
-        <v>2.8</v>
+      <c r="F59" s="1" t="n"/>
+      <c r="G59" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>4.083333333333333</v>
       </c>
     </row>
     <row r="60">
@@ -1418,13 +1489,14 @@
       <c r="C60" s="1" t="n"/>
       <c r="D60" s="1" t="n"/>
       <c r="E60" s="1" t="n"/>
-      <c r="F60" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>3.8</v>
+      <c r="F60" s="1" t="n"/>
+      <c r="G60" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>4.583333333333333</v>
       </c>
     </row>
     <row r="61">
@@ -1433,19 +1505,20 @@
       <c r="C61" s="1" t="n"/>
       <c r="D61" s="1" t="n"/>
       <c r="E61" s="1" t="n"/>
-      <c r="F61" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_single_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>2.8</v>
+      <c r="F61" s="1" t="n"/>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_ga_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>Varying</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="B62" s="1" t="n">
@@ -1453,24 +1526,29 @@
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="inlineStr">
+        <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D62" s="1" t="inlineStr">
+      <c r="E62" s="1" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E62" s="1" t="n">
+      <c r="F62" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F62" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>4.3</v>
+      <c r="G62" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>1.916666666666667</v>
       </c>
     </row>
     <row r="63">
@@ -1479,13 +1557,14 @@
       <c r="C63" s="1" t="n"/>
       <c r="D63" s="1" t="n"/>
       <c r="E63" s="1" t="n"/>
-      <c r="F63" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>4.5</v>
+      <c r="F63" s="1" t="n"/>
+      <c r="G63" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -1494,13 +1573,14 @@
       <c r="C64" s="1" t="n"/>
       <c r="D64" s="1" t="n"/>
       <c r="E64" s="1" t="n"/>
-      <c r="F64" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>4.6</v>
+      <c r="F64" s="1" t="n"/>
+      <c r="G64" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -1509,13 +1589,14 @@
       <c r="C65" s="1" t="n"/>
       <c r="D65" s="1" t="n"/>
       <c r="E65" s="1" t="n"/>
-      <c r="F65" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G65" t="n">
-        <v>4.6</v>
+      <c r="F65" s="1" t="n"/>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -1524,13 +1605,14 @@
       <c r="C66" s="1" t="n"/>
       <c r="D66" s="1" t="n"/>
       <c r="E66" s="1" t="n"/>
-      <c r="F66" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G66" t="n">
-        <v>4.6</v>
+      <c r="F66" s="1" t="n"/>
+      <c r="G66" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="67">
@@ -1539,13 +1621,14 @@
       <c r="C67" s="1" t="n"/>
       <c r="D67" s="1" t="n"/>
       <c r="E67" s="1" t="n"/>
-      <c r="F67" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G67" t="n">
-        <v>4.4</v>
+      <c r="F67" s="1" t="n"/>
+      <c r="G67" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="68">
@@ -1554,13 +1637,14 @@
       <c r="C68" s="1" t="n"/>
       <c r="D68" s="1" t="n"/>
       <c r="E68" s="1" t="n"/>
-      <c r="F68" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G68" t="n">
-        <v>4.2</v>
+      <c r="F68" s="1" t="n"/>
+      <c r="G68" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>1.916666666666667</v>
       </c>
     </row>
     <row r="69">
@@ -1569,13 +1653,14 @@
       <c r="C69" s="1" t="n"/>
       <c r="D69" s="1" t="n"/>
       <c r="E69" s="1" t="n"/>
-      <c r="F69" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G69" t="n">
-        <v>4.4</v>
+      <c r="F69" s="1" t="n"/>
+      <c r="G69" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -1584,13 +1669,14 @@
       <c r="C70" s="1" t="n"/>
       <c r="D70" s="1" t="n"/>
       <c r="E70" s="1" t="n"/>
-      <c r="F70" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G70" t="n">
-        <v>4.7</v>
+      <c r="F70" s="1" t="n"/>
+      <c r="G70" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -1599,34 +1685,36 @@
       <c r="C71" s="1" t="n"/>
       <c r="D71" s="1" t="n"/>
       <c r="E71" s="1" t="n"/>
-      <c r="F71" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_varying_sliced_10.ini</t>
-        </is>
-      </c>
-      <c r="G71" t="n">
-        <v>4.1</v>
+      <c r="F71" s="1" t="n"/>
+      <c r="G71" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_single_sliced_10.ini</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n"/>
       <c r="B72" s="1" t="n"/>
       <c r="C72" s="1" t="n"/>
-      <c r="D72" s="1" t="inlineStr">
+      <c r="D72" s="1" t="n"/>
+      <c r="E72" s="1" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E72" s="1" t="n">
+      <c r="F72" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F72" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G72" t="n">
-        <v>6.4</v>
+      <c r="G72" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>1.916666666666667</v>
       </c>
     </row>
     <row r="73">
@@ -1635,13 +1723,14 @@
       <c r="C73" s="1" t="n"/>
       <c r="D73" s="1" t="n"/>
       <c r="E73" s="1" t="n"/>
-      <c r="F73" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G73" t="n">
-        <v>6.5</v>
+      <c r="F73" s="1" t="n"/>
+      <c r="G73" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="74">
@@ -1650,13 +1739,14 @@
       <c r="C74" s="1" t="n"/>
       <c r="D74" s="1" t="n"/>
       <c r="E74" s="1" t="n"/>
-      <c r="F74" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G74" t="n">
-        <v>6</v>
+      <c r="F74" s="1" t="n"/>
+      <c r="G74" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="75">
@@ -1665,13 +1755,14 @@
       <c r="C75" s="1" t="n"/>
       <c r="D75" s="1" t="n"/>
       <c r="E75" s="1" t="n"/>
-      <c r="F75" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G75" t="n">
-        <v>6.6</v>
+      <c r="F75" s="1" t="n"/>
+      <c r="G75" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -1680,13 +1771,14 @@
       <c r="C76" s="1" t="n"/>
       <c r="D76" s="1" t="n"/>
       <c r="E76" s="1" t="n"/>
-      <c r="F76" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G76" t="n">
-        <v>6.2</v>
+      <c r="F76" s="1" t="n"/>
+      <c r="G76" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="77">
@@ -1695,13 +1787,14 @@
       <c r="C77" s="1" t="n"/>
       <c r="D77" s="1" t="n"/>
       <c r="E77" s="1" t="n"/>
-      <c r="F77" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G77" t="n">
-        <v>6.4</v>
+      <c r="F77" s="1" t="n"/>
+      <c r="G77" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>1.916666666666667</v>
       </c>
     </row>
     <row r="78">
@@ -1710,13 +1803,14 @@
       <c r="C78" s="1" t="n"/>
       <c r="D78" s="1" t="n"/>
       <c r="E78" s="1" t="n"/>
-      <c r="F78" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G78" t="n">
-        <v>6.5</v>
+      <c r="F78" s="1" t="n"/>
+      <c r="G78" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>1.916666666666667</v>
       </c>
     </row>
     <row r="79">
@@ -1725,13 +1819,14 @@
       <c r="C79" s="1" t="n"/>
       <c r="D79" s="1" t="n"/>
       <c r="E79" s="1" t="n"/>
-      <c r="F79" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G79" t="n">
-        <v>6.6</v>
+      <c r="F79" s="1" t="n"/>
+      <c r="G79" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -1740,13 +1835,14 @@
       <c r="C80" s="1" t="n"/>
       <c r="D80" s="1" t="n"/>
       <c r="E80" s="1" t="n"/>
-      <c r="F80" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G80" t="n">
-        <v>6.4</v>
+      <c r="F80" s="1" t="n"/>
+      <c r="G80" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="81">
@@ -1755,34 +1851,36 @@
       <c r="C81" s="1" t="n"/>
       <c r="D81" s="1" t="n"/>
       <c r="E81" s="1" t="n"/>
-      <c r="F81" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_varying_sliced_15.ini</t>
-        </is>
-      </c>
-      <c r="G81" t="n">
-        <v>5.9</v>
+      <c r="F81" s="1" t="n"/>
+      <c r="G81" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_single_sliced_15.ini</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n"/>
       <c r="B82" s="1" t="n"/>
       <c r="C82" s="1" t="n"/>
-      <c r="D82" s="1" t="inlineStr">
+      <c r="D82" s="1" t="n"/>
+      <c r="E82" s="1" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E82" s="1" t="n">
+      <c r="F82" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F82" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G82" t="n">
-        <v>3.3</v>
+      <c r="G82" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_10/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -1791,13 +1889,14 @@
       <c r="C83" s="1" t="n"/>
       <c r="D83" s="1" t="n"/>
       <c r="E83" s="1" t="n"/>
-      <c r="F83" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G83" t="n">
-        <v>3.2</v>
+      <c r="F83" s="1" t="n"/>
+      <c r="G83" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_11/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -1806,13 +1905,14 @@
       <c r="C84" s="1" t="n"/>
       <c r="D84" s="1" t="n"/>
       <c r="E84" s="1" t="n"/>
-      <c r="F84" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G84" t="n">
-        <v>3</v>
+      <c r="F84" s="1" t="n"/>
+      <c r="G84" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_12/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -1821,13 +1921,14 @@
       <c r="C85" s="1" t="n"/>
       <c r="D85" s="1" t="n"/>
       <c r="E85" s="1" t="n"/>
-      <c r="F85" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G85" t="n">
-        <v>3.3</v>
+      <c r="F85" s="1" t="n"/>
+      <c r="G85" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_13/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -1836,13 +1937,14 @@
       <c r="C86" s="1" t="n"/>
       <c r="D86" s="1" t="n"/>
       <c r="E86" s="1" t="n"/>
-      <c r="F86" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G86" t="n">
-        <v>3.3</v>
+      <c r="F86" s="1" t="n"/>
+      <c r="G86" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_2/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>2.833333333333333</v>
       </c>
     </row>
     <row r="87">
@@ -1851,13 +1953,14 @@
       <c r="C87" s="1" t="n"/>
       <c r="D87" s="1" t="n"/>
       <c r="E87" s="1" t="n"/>
-      <c r="F87" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G87" t="n">
-        <v>3.1</v>
+      <c r="F87" s="1" t="n"/>
+      <c r="G87" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_3/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="88">
@@ -1866,13 +1969,14 @@
       <c r="C88" s="1" t="n"/>
       <c r="D88" s="1" t="n"/>
       <c r="E88" s="1" t="n"/>
-      <c r="F88" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G88" t="n">
-        <v>3.4</v>
+      <c r="F88" s="1" t="n"/>
+      <c r="G88" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_4/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>1.916666666666667</v>
       </c>
     </row>
     <row r="89">
@@ -1881,13 +1985,14 @@
       <c r="C89" s="1" t="n"/>
       <c r="D89" s="1" t="n"/>
       <c r="E89" s="1" t="n"/>
-      <c r="F89" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G89" t="n">
-        <v>3.2</v>
+      <c r="F89" s="1" t="n"/>
+      <c r="G89" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -1896,13 +2001,14 @@
       <c r="C90" s="1" t="n"/>
       <c r="D90" s="1" t="n"/>
       <c r="E90" s="1" t="n"/>
-      <c r="F90" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G90" t="n">
-        <v>3.3</v>
+      <c r="F90" s="1" t="n"/>
+      <c r="G90" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -1911,17 +2017,18 @@
       <c r="C91" s="1" t="n"/>
       <c r="D91" s="1" t="n"/>
       <c r="E91" s="1" t="n"/>
-      <c r="F91" s="1" t="inlineStr">
-        <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_varying_sliced_5.ini</t>
-        </is>
-      </c>
-      <c r="G91" t="n">
-        <v>2.8</v>
+      <c r="F91" s="1" t="n"/>
+      <c r="G91" s="1" t="inlineStr">
+        <is>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_7/ilp_single_sliced_5.ini</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="30">
     <mergeCell ref="A2:A31"/>
     <mergeCell ref="A32:A61"/>
     <mergeCell ref="A62:A91"/>
@@ -1931,15 +2038,9 @@
     <mergeCell ref="C2:C31"/>
     <mergeCell ref="C32:C61"/>
     <mergeCell ref="C62:C91"/>
-    <mergeCell ref="D2:D11"/>
-    <mergeCell ref="D12:D21"/>
-    <mergeCell ref="D22:D31"/>
-    <mergeCell ref="D32:D41"/>
-    <mergeCell ref="D42:D51"/>
-    <mergeCell ref="D52:D61"/>
-    <mergeCell ref="D62:D71"/>
-    <mergeCell ref="D72:D81"/>
-    <mergeCell ref="D82:D91"/>
+    <mergeCell ref="D2:D31"/>
+    <mergeCell ref="D32:D61"/>
+    <mergeCell ref="D62:D91"/>
     <mergeCell ref="E2:E11"/>
     <mergeCell ref="E12:E21"/>
     <mergeCell ref="E22:E31"/>
@@ -1949,6 +2050,15 @@
     <mergeCell ref="E62:E71"/>
     <mergeCell ref="E72:E81"/>
     <mergeCell ref="E82:E91"/>
+    <mergeCell ref="F2:F11"/>
+    <mergeCell ref="F12:F21"/>
+    <mergeCell ref="F22:F31"/>
+    <mergeCell ref="F32:F41"/>
+    <mergeCell ref="F42:F51"/>
+    <mergeCell ref="F52:F61"/>
+    <mergeCell ref="F62:F71"/>
+    <mergeCell ref="F72:F81"/>
+    <mergeCell ref="F82:F91"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pushing results file and log
</commit_message>
<xml_diff>
--- a/Functions/Images/disaster_percentage_0/micro_power_30/enb_data.xlsx
+++ b/Functions/Images/disaster_percentage_0/micro_power_30/enb_data.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="ILPCompare" sheetId="1" state="visible" r:id="rId1"/>
@@ -74,18 +74,18 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -494,7 +494,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Gwo</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -520,11 +520,11 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_fixed_sliced_10.ini</t>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_gwo_sliced_10.ini</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>4.666666666666667</v>
+        <v>6.083333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -536,11 +536,11 @@
       <c r="F3" s="1" t="n"/>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_fixed_sliced_10.ini</t>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_gwo_sliced_10.ini</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>4.75</v>
+        <v>5.666666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -558,11 +558,11 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_fixed_sliced_15.ini</t>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_gwo_sliced_15.ini</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>7.333333333333333</v>
+        <v>8.833333333333334</v>
       </c>
     </row>
     <row r="5">
@@ -574,11 +574,11 @@
       <c r="F5" s="1" t="n"/>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_fixed_sliced_15.ini</t>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_gwo_sliced_15.ini</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>7.5</v>
+        <v>8.416666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -596,11 +596,11 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_fixed_sliced_5.ini</t>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_5/ilp_gwo_sliced_5.ini</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3.666666666666667</v>
+        <v>4.916666666666667</v>
       </c>
     </row>
     <row r="7">
@@ -612,11 +612,11 @@
       <c r="F7" s="1" t="n"/>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_fixed_sliced_5.ini</t>
+          <t>../Network_CCOpMv/_5G/simulations/disaster_percentage_0/micro_power_30/chosen_seed_6/ilp_gwo_sliced_5.ini</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>3.666666666666667</v>
+        <v>5.333333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -632,6 +632,6 @@
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="F6:F7"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>